<commit_message>
Renamed files and added defects to requirements and architecture.
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\negre\MyDrinkShop\docs\Lab01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alle\IdeaProjects\VVSS\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89567E27-6FC5-4B76-9816-C9E61DC4A70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="23040" windowHeight="13560" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="23040" windowHeight="13560" tabRatio="650" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="1" r:id="rId1"/>
@@ -18,7 +17,7 @@
     <sheet name="Coding Phase Defects" sheetId="3" r:id="rId3"/>
     <sheet name="Tool-basedCodeAnalysis" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="102">
   <si>
     <t>do not print this form</t>
   </si>
@@ -140,18 +139,12 @@
     <t>A05</t>
   </si>
   <si>
-    <t>Diagram_v1.0, toate clasele</t>
-  </si>
-  <si>
     <t>Nu exista o strategie coerenta de tratare a erorilor reflectata in diagrama. ValidationException exista in cod dar nu apare in diagrama, si nu este definit un mecanism centralizat de error handling la nivel arhitectural.</t>
   </si>
   <si>
     <t>A03</t>
   </si>
   <si>
-    <t>Diagram_v1.0</t>
-  </si>
-  <si>
     <t>Diagrama nu include clase Repository pentru TipBautura si CategorieBautura, desi cerinta 3 specifica explicit CRUD pentru aceste entitati. Arhitectura nu acopera toate cerintele functionale.</t>
   </si>
   <si>
@@ -164,21 +157,12 @@
     <t>A07</t>
   </si>
   <si>
-    <t>Diagram_v1.0, clasa DrinkShopService</t>
-  </si>
-  <si>
     <t>Clasa DrinkShopService functioneaza ca un Facade, dar rolul sau nu este explicit documentat in diagrama. Descrierea clasei nu mentioneaza responsabilitatea de coordonare a serviciilor.</t>
   </si>
   <si>
     <t>A09</t>
   </si>
   <si>
-    <t>Diagram_v1.0, Order-OrderItem, Reteta-IngredientReteta</t>
-  </si>
-  <si>
-    <t>Relatiile de asociere/agregare din diagrama nu au multiplicitate definita. Ex: Order-OrderItem (1..*), Reteta-IngredientReteta (1..*) - informatii absente din diagrama curenta.</t>
-  </si>
-  <si>
     <t>Review Form. Coding Defects</t>
   </si>
   <si>
@@ -305,9 +289,6 @@
     <t>1.0</t>
   </si>
   <si>
-    <t>a</t>
-  </si>
-  <si>
     <t>Negrea Razvan</t>
   </si>
   <si>
@@ -318,12 +299,57 @@
   </si>
   <si>
     <t>Nagel Roland</t>
+  </si>
+  <si>
+    <t>Requirements_v1.0.pdf, p.1, cerința 2</t>
+  </si>
+  <si>
+    <t>Nu se specifică diferența dintre tip și categorie, respectiv ce ar trebui să reprezinte acestea.</t>
+  </si>
+  <si>
+    <t>R04</t>
+  </si>
+  <si>
+    <t>Nu se specifică ce ar trebui să facă aplicația în cazul în care fișierele de persistență a datelor sunt corupte/prost formatate.</t>
+  </si>
+  <si>
+    <t>Nu se specifică ce ar trebui să conțină ecranul de pornire și dacă comenzile anterioare ar trebui încărcate.</t>
+  </si>
+  <si>
+    <t>Requirements_v1.0.pdf, p., cerința 8</t>
+  </si>
+  <si>
+    <t>Nu se menționează ce se întâmplă în cazul închiderii aplicației înainte de salvarea comenzilor pentru ziua curentă.</t>
+  </si>
+  <si>
+    <t>Requirements_MyDrinkShop.png_1.1.png, toate clasele</t>
+  </si>
+  <si>
+    <t>Requirements_MyDrinkShop.png_1.1.png</t>
+  </si>
+  <si>
+    <t>Requirements_MyDrinkShop.png_1.1.png, clasa DrinkShopService</t>
+  </si>
+  <si>
+    <t>Requirements_MyDrinkShop.png_1.1.pn, clasa DrinkShopApp</t>
+  </si>
+  <si>
+    <t>Clasa DrinkShopApp nu este asociată cu DrinkShopControlle, deși se folosește de aceasta.</t>
+  </si>
+  <si>
+    <t>A01</t>
+  </si>
+  <si>
+    <t>Requirements_MyDrinkShop.png_1.1.png, clasa ProductTest</t>
+  </si>
+  <si>
+    <t>Fișierele de test nu ar trebui incluse în diagrama.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -523,7 +549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -542,9 +568,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -601,6 +624,16 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -619,9 +652,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -659,9 +692,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -696,7 +729,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -731,7 +764,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -904,7 +937,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
@@ -913,7 +946,8 @@
   <cols>
     <col min="1" max="1" width="8.88671875" style="6" customWidth="1"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.21875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="32.77734375" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
     <col min="6" max="8" width="8.88671875" style="6" customWidth="1"/>
     <col min="9" max="9" width="21" style="6" customWidth="1"/>
@@ -927,35 +961,35 @@
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="30"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="16" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="27" t="s">
-        <v>89</v>
-      </c>
-      <c r="J3" s="17">
+      <c r="I3" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="J3" s="16">
         <v>234</v>
       </c>
     </row>
@@ -963,15 +997,15 @@
       <c r="C4" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="D4" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="30"/>
-      <c r="H4" s="17" t="s">
+      <c r="E4" s="29"/>
+      <c r="H4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="27" t="s">
-        <v>92</v>
+      <c r="I4" s="26" t="s">
+        <v>86</v>
       </c>
       <c r="J4" s="3">
         <v>234</v>
@@ -981,15 +1015,15 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" s="30"/>
-      <c r="H5" s="17" t="s">
+      <c r="D5" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="29"/>
+      <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="27" t="s">
-        <v>91</v>
+      <c r="I5" s="26" t="s">
+        <v>85</v>
       </c>
       <c r="J5" s="3">
         <v>234</v>
@@ -1000,19 +1034,19 @@
       <c r="C6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="31" t="s">
+      <c r="D7" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="29"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1023,18 +1057,16 @@
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="22" t="s">
-        <v>88</v>
-      </c>
+      <c r="G10" s="21"/>
     </row>
     <row r="11" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
@@ -1081,41 +1113,65 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="2"/>
+      <c r="C17" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="3">
@@ -1124,7 +1180,7 @@
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
-      <c r="E18" s="15"/>
+      <c r="E18" s="14"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="3">
@@ -1133,7 +1189,7 @@
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
-      <c r="E19" s="15"/>
+      <c r="E19" s="14"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
@@ -1142,7 +1198,7 @@
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
-      <c r="E20" s="15"/>
+      <c r="E20" s="14"/>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="3">
@@ -1151,7 +1207,7 @@
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
-      <c r="E21" s="15"/>
+      <c r="E21" s="14"/>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="3">
@@ -1160,7 +1216,7 @@
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
-      <c r="E22" s="15"/>
+      <c r="E22" s="14"/>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="3">
@@ -1169,7 +1225,7 @@
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
-      <c r="E23" s="15"/>
+      <c r="E23" s="14"/>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="3">
@@ -1178,7 +1234,7 @@
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
-      <c r="E24" s="15"/>
+      <c r="E24" s="14"/>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="3">
@@ -1187,19 +1243,19 @@
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
-      <c r="E25" s="15"/>
+      <c r="E25" s="14"/>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D26" t="s">
-        <v>27</v>
-      </c>
+      <c r="D26"/>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C27" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D27" s="12"/>
-      <c r="E27" s="1"/>
+      <c r="E27" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1216,7 +1272,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
@@ -1225,7 +1281,8 @@
   <cols>
     <col min="1" max="1" width="8.88671875" style="6" customWidth="1"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.21875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="73.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
     <col min="6" max="8" width="8.88671875" style="6" customWidth="1"/>
     <col min="9" max="9" width="22.109375" style="6" customWidth="1"/>
@@ -1238,35 +1295,35 @@
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="30"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="16" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="27" t="s">
-        <v>91</v>
-      </c>
-      <c r="J3" s="17">
+      <c r="I3" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="J3" s="16">
         <v>234</v>
       </c>
     </row>
@@ -1274,15 +1331,15 @@
       <c r="C4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="30"/>
-      <c r="H4" s="17" t="s">
+      <c r="E4" s="29"/>
+      <c r="H4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="27" t="s">
-        <v>90</v>
+      <c r="I4" s="26" t="s">
+        <v>84</v>
       </c>
       <c r="J4" s="3">
         <v>234</v>
@@ -1292,15 +1349,15 @@
       <c r="C5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" s="30"/>
-      <c r="H5" s="17" t="s">
+      <c r="D5" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="29"/>
+      <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="27" t="s">
-        <v>89</v>
+      <c r="I5" s="26" t="s">
+        <v>83</v>
       </c>
       <c r="J5" s="3">
         <v>234</v>
@@ -1311,37 +1368,40 @@
       <c r="C6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="31" t="s">
+      <c r="D7" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="29"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="43" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" s="42" t="s">
         <v>33</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="72" x14ac:dyDescent="0.3">
@@ -1350,13 +1410,13 @@
         <v>2</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
@@ -1365,43 +1425,43 @@
         <v>3</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="3">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="D13" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B13" s="3">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="C13" s="1" t="s">
+    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B14" s="3">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B14" s="3">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="D14" s="1" t="s">
-        <v>44</v>
+        <v>97</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>45</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -1409,9 +1469,15 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="2"/>
+      <c r="C15" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
@@ -1513,16 +1579,16 @@
       <c r="E26" s="2"/>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D27" t="s">
-        <v>27</v>
-      </c>
+      <c r="D27"/>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C28" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D28" s="12"/>
-      <c r="E28" s="1"/>
+      <c r="E28" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1539,7 +1605,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
@@ -1549,7 +1615,7 @@
     <col min="1" max="1" width="8.88671875" style="6" customWidth="1"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
     <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
+    <col min="4" max="4" width="30" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
     <col min="6" max="8" width="8.88671875" style="6" customWidth="1"/>
     <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
@@ -1562,69 +1628,69 @@
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="30"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
+      <c r="B2" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="16" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="27" t="s">
-        <v>92</v>
-      </c>
-      <c r="J3" s="17">
+      <c r="I3" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="J3" s="16">
         <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="39" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="30"/>
-      <c r="H4" s="17" t="s">
+      <c r="D4" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="29"/>
+      <c r="H4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="27" t="s">
-        <v>91</v>
+      <c r="I4" s="26" t="s">
+        <v>85</v>
       </c>
       <c r="J4" s="3">
         <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="38" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" s="30"/>
-      <c r="H5" s="17" t="s">
+      <c r="D5" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="29"/>
+      <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="27" t="s">
-        <v>89</v>
+      <c r="I5" s="26" t="s">
+        <v>83</v>
       </c>
       <c r="J5" s="3">
         <v>234</v>
@@ -1635,37 +1701,40 @@
       <c r="C6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="31" t="s">
+      <c r="D7" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="29"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>50</v>
+      <c r="C10" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="72" x14ac:dyDescent="0.3">
@@ -1674,13 +1743,13 @@
         <v>2</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
@@ -1689,13 +1758,13 @@
         <v>3</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
@@ -1704,13 +1773,13 @@
         <v>4</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="72" x14ac:dyDescent="0.3">
@@ -1719,13 +1788,13 @@
         <v>5</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -1899,7 +1968,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
@@ -1923,51 +1992,51 @@
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="30"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
+      <c r="B2" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="16" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="27" t="s">
-        <v>91</v>
-      </c>
-      <c r="J3" s="17">
+      <c r="I3" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="J3" s="16">
         <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C4" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="D4" s="39" t="s">
-        <v>65</v>
-      </c>
-      <c r="E4" s="30"/>
-      <c r="H4" s="17" t="s">
+      <c r="C4" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="29"/>
+      <c r="H4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="27" t="s">
-        <v>92</v>
+      <c r="I4" s="26" t="s">
+        <v>86</v>
       </c>
       <c r="J4" s="3">
         <v>234</v>
@@ -1977,15 +2046,15 @@
       <c r="C5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="30"/>
-      <c r="H5" s="17" t="s">
+      <c r="E5" s="29"/>
+      <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="27" t="s">
-        <v>89</v>
+      <c r="I5" s="26" t="s">
+        <v>83</v>
       </c>
       <c r="J5" s="3">
         <v>234</v>
@@ -1996,50 +2065,54 @@
       <c r="C6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="30"/>
-      <c r="F6" s="20"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="19"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" t="s">
-        <v>67</v>
-      </c>
-      <c r="E10" t="s">
-        <v>68</v>
-      </c>
-      <c r="F10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="112.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="40" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" s="41" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" s="41" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <f t="shared" ref="B11:B30" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>73</v>
+      <c r="C11" s="42" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="42" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="42" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -2047,17 +2120,17 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="E12" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="F12" s="26" t="s">
-        <v>77</v>
+      <c r="C12" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="F12" s="25" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -2065,17 +2138,17 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="E13" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="F13" s="26" t="s">
-        <v>81</v>
+      <c r="C13" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -2083,17 +2156,17 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="D14" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="E14" s="26" t="s">
-        <v>84</v>
-      </c>
-      <c r="F14" s="26" t="s">
-        <v>85</v>
+      <c r="C14" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="25" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -2257,20 +2330,20 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="40" t="s">
-        <v>86</v>
-      </c>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="18"/>
+      <c r="C32" s="39" t="s">
+        <v>81</v>
+      </c>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="17"/>
     </row>
     <row r="34" spans="4:6" x14ac:dyDescent="0.3">
       <c r="D34" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="35" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="F35" s="21"/>
+      <c r="F35" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2283,6 +2356,6 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add changes and new files
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alle\IdeaProjects\VVSS\docs\Lab01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VVSS\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74583BC7-1B3F-4C0F-92B3-45554EE1BC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="23040" windowHeight="13560" tabRatio="650" activeTab="1"/>
+    <workbookView xWindow="3375" yWindow="1260" windowWidth="28800" windowHeight="15345" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="1" r:id="rId1"/>
@@ -17,19 +18,8 @@
     <sheet name="Coding Phase Defects" sheetId="3" r:id="rId3"/>
     <sheet name="Tool-basedCodeAnalysis" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -349,7 +339,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -591,6 +581,16 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -624,16 +624,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -652,9 +642,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -692,9 +682,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -729,7 +719,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -764,7 +754,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -937,43 +927,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="32.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.88671875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6" customWidth="1"/>
     <col min="9" max="9" width="21" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="8.88671875" style="6" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
+    <col min="10" max="10" width="14.42578125" style="6" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" style="6" customWidth="1"/>
+    <col min="12" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="I1" s="32"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
       <c r="H2" s="3"/>
       <c r="I2" s="18" t="s">
         <v>3</v>
@@ -982,7 +972,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
@@ -993,14 +983,14 @@
         <v>234</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
       </c>
@@ -1011,14 +1001,14 @@
         <v>234</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="35" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="29"/>
+      <c r="E5" s="33"/>
       <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
@@ -1029,31 +1019,31 @@
         <v>234</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="29"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E6" s="33"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="29"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E7" s="33"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1068,7 +1058,7 @@
       </c>
       <c r="G10" s="21"/>
     </row>
-    <row r="11" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f t="shared" ref="B11:B25" si="0">B10+1</f>
         <v>2</v>
@@ -1083,7 +1073,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1098,7 +1088,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1113,7 +1103,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1128,7 +1118,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1143,7 +1133,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1158,7 +1148,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1173,7 +1163,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1182,7 +1172,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="14"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1191,7 +1181,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="14"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1200,7 +1190,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="14"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1209,7 +1199,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="14"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1218,7 +1208,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="14"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1227,7 +1217,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="14"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1236,7 +1226,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="14"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1245,10 +1235,10 @@
       <c r="D25" s="3"/>
       <c r="E25" s="14"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D26"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C27" s="11" t="s">
         <v>28</v>
       </c>
@@ -1272,42 +1262,42 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="73.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.88671875" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.109375" style="6" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="73.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="22.140625" style="6" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="I1" s="32"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
       <c r="H2" s="3"/>
       <c r="I2" s="18" t="s">
         <v>3</v>
@@ -1316,7 +1306,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
@@ -1327,14 +1317,14 @@
         <v>234</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
       </c>
@@ -1345,14 +1335,14 @@
         <v>234</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="39" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="29"/>
+      <c r="E5" s="33"/>
       <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
@@ -1363,26 +1353,26 @@
         <v>234</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="29"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E6" s="33"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="29"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E7" s="33"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>15</v>
       </c>
@@ -1390,21 +1380,21 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="43" t="s">
+      <c r="D10" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="E10" s="42" t="s">
+      <c r="E10" s="29" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f t="shared" ref="B11:B26" si="0">B10+1</f>
         <v>2</v>
@@ -1419,7 +1409,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1434,7 +1424,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1449,7 +1439,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1464,7 +1454,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1479,7 +1469,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1488,7 +1478,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1497,7 +1487,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1506,7 +1496,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1515,7 +1505,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1524,7 +1514,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1533,7 +1523,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1542,7 +1532,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1551,7 +1541,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1560,7 +1550,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1569,7 +1559,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1578,10 +1568,10 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D27"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C28" s="11" t="s">
         <v>28</v>
       </c>
@@ -1605,42 +1595,42 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
     <col min="4" max="4" width="30" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.88671875" style="6" customWidth="1"/>
-    <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="I1" s="32"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
       <c r="H2" s="3"/>
       <c r="I2" s="18" t="s">
         <v>3</v>
@@ -1649,7 +1639,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
@@ -1660,14 +1650,14 @@
         <v>234</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
       </c>
@@ -1678,14 +1668,14 @@
         <v>234</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="29"/>
+      <c r="E5" s="33"/>
       <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
@@ -1696,26 +1686,26 @@
         <v>234</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="29"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E6" s="33"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="29"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E7" s="33"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>15</v>
       </c>
@@ -1723,21 +1713,21 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="42" t="s">
+      <c r="D10" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="42" t="s">
+      <c r="E10" s="29" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f t="shared" ref="B11:B30" si="0">B10+1</f>
         <v>2</v>
@@ -1752,7 +1742,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1767,7 +1757,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1782,7 +1772,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1797,7 +1787,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1806,7 +1796,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1815,7 +1805,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1824,7 +1814,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1833,7 +1823,7 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1842,7 +1832,7 @@
       <c r="D19" s="1"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1851,7 +1841,7 @@
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1860,7 +1850,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1869,7 +1859,7 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1878,7 +1868,7 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1887,7 +1877,7 @@
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1896,7 +1886,7 @@
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1905,7 +1895,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1914,7 +1904,7 @@
       <c r="D27" s="2"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1923,7 +1913,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1932,7 +1922,7 @@
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1941,12 +1931,12 @@
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C32" s="11" t="s">
         <v>28</v>
       </c>
@@ -1968,43 +1958,43 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="37.44140625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="37.5546875" style="6" customWidth="1"/>
-    <col min="5" max="5" width="36.21875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="48.6640625" style="6" customWidth="1"/>
-    <col min="7" max="8" width="8.88671875" style="6" customWidth="1"/>
-    <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="37.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="36.28515625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="48.7109375" style="6" customWidth="1"/>
+    <col min="7" max="8" width="8.85546875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="I1" s="32"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="37" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
       <c r="H2" s="3"/>
       <c r="I2" s="18" t="s">
         <v>3</v>
@@ -2013,7 +2003,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
@@ -2024,14 +2014,14 @@
         <v>234</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
       </c>
@@ -2042,14 +2032,14 @@
         <v>234</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="29"/>
+      <c r="E5" s="33"/>
       <c r="H5" s="16" t="s">
         <v>10</v>
       </c>
@@ -2060,18 +2050,18 @@
         <v>234</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="29"/>
+      <c r="E6" s="33"/>
       <c r="F6" s="19"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2080,42 +2070,42 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="40" t="s">
+      <c r="C10" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="28" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f t="shared" ref="B11:B30" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="42" t="s">
+      <c r="D11" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="F11" s="42" t="s">
+      <c r="F11" s="29" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -2133,7 +2123,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2151,7 +2141,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2169,7 +2159,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2179,7 +2169,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2189,7 +2179,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2199,7 +2189,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2209,7 +2199,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2219,7 +2209,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2229,7 +2219,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2239,7 +2229,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2249,7 +2239,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2259,7 +2249,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2269,7 +2259,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2279,7 +2269,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2289,7 +2279,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2299,7 +2289,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2309,7 +2299,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2319,7 +2309,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2329,20 +2319,20 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="39" t="s">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C32" s="43" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
       <c r="F32" s="17"/>
     </row>
-    <row r="34" spans="4:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="35" spans="4:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F35" s="20"/>
     </row>
   </sheetData>

</xml_diff>